<commit_message>
r sheets + added video
</commit_message>
<xml_diff>
--- a/0-course-info/canvas/canvas_schedule.xlsx
+++ b/0-course-info/canvas/canvas_schedule.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/0-course-info/canvas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31CE0D9C-0407-FC42-8240-BF3272928C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95DA8F0-5993-7249-84F8-020AE45CE11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="27240" windowHeight="16180" xr2:uid="{BA0A3FFF-9577-8249-B793-6919848B638A}"/>
+    <workbookView xWindow="17740" yWindow="-18800" windowWidth="27240" windowHeight="16180" xr2:uid="{BA0A3FFF-9577-8249-B793-6919848B638A}"/>
   </bookViews>
   <sheets>
-    <sheet name="schedule" sheetId="1" r:id="rId1"/>
+    <sheet name="schedule" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="67">
   <si>
     <t>Week</t>
   </si>
@@ -76,10 +76,6 @@
   </si>
   <si>
     <t>Th</t>
-  </si>
-  <si>
-    <t>Syllabus quiz + intro survey
-Lecture Video: Controlling for Variability</t>
   </si>
   <si>
     <t>Activity 1.2 + Start Lab 1</t>
@@ -104,9 +100,6 @@
     <t>Activity 2.2</t>
   </si>
   <si>
-    <t>Lab 1 due 9/4</t>
-  </si>
-  <si>
     <t>Mod 3: Power and Sample Size</t>
   </si>
   <si>
@@ -248,13 +241,17 @@
     <t>SEC X02 Final Exam 10:00 - 12:30</t>
   </si>
   <si>
-    <t>Lab 5 due 11/20</t>
-  </si>
-  <si>
-    <t>Start Lab 5</t>
-  </si>
-  <si>
-    <t>Lab 4 due 10/30</t>
+    <t>Discord and R / Rstudio Setup
+Lecture Video: Controlling for Variability</t>
+  </si>
+  <si>
+    <t>Lab Group Contract due 8/30</t>
+  </si>
+  <si>
+    <t>Lab 1 due 9/8</t>
+  </si>
+  <si>
+    <t>Lab 4 due 11/20</t>
   </si>
 </sst>
 </file>
@@ -264,7 +261,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -298,12 +295,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -370,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -510,11 +501,20 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -527,18 +527,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -873,7 +861,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9F0D472-3E01-A348-B672-A72D1DCE07F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{764FB71E-3535-E54A-BA2B-188557212004}">
   <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -912,7 +900,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" s="47">
+      <c r="A2" s="49">
         <v>1</v>
       </c>
       <c r="B2" s="4">
@@ -935,7 +923,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="47"/>
+      <c r="A3" s="49"/>
       <c r="B3" s="4">
         <v>2</v>
       </c>
@@ -950,24 +938,26 @@
         <v>8</v>
       </c>
       <c r="F3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="48"/>
+      <c r="A4" s="50"/>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
       <c r="E4" s="12"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
+      <c r="H4" s="14" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A5" s="53">
+      <c r="A5" s="48">
         <v>2</v>
       </c>
       <c r="B5" s="15">
@@ -982,18 +972,18 @@
         <v>46266</v>
       </c>
       <c r="E5" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="G5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>16</v>
-      </c>
       <c r="H5" s="19"/>
     </row>
     <row r="6" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A6" s="47"/>
+      <c r="A6" s="49"/>
       <c r="B6" s="4">
         <f>B5+1</f>
         <v>4</v>
@@ -1006,29 +996,27 @@
         <v>46268</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="7" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="48"/>
+      <c r="A7" s="50"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="11"/>
       <c r="E7" s="12"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
-      <c r="H7" s="14" t="s">
-        <v>19</v>
-      </c>
+      <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="47">
+      <c r="A8" s="49">
         <v>3</v>
       </c>
       <c r="B8" s="4">
@@ -1043,17 +1031,20 @@
         <v>46273</v>
       </c>
       <c r="E8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>22</v>
+      <c r="H8" s="8" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="47"/>
+      <c r="A9" s="49"/>
       <c r="B9" s="4">
         <f>B8+1</f>
         <v>6</v>
@@ -1066,17 +1057,17 @@
         <v>46275</v>
       </c>
       <c r="E9" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G9" t="s">
         <v>23</v>
       </c>
-      <c r="F9" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="10" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="48"/>
+      <c r="A10" s="50"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="11"/>
@@ -1086,7 +1077,7 @@
       <c r="H10" s="14"/>
     </row>
     <row r="11" spans="1:8" ht="32" x14ac:dyDescent="0.2">
-      <c r="A11" s="53">
+      <c r="A11" s="48">
         <v>4</v>
       </c>
       <c r="B11" s="15">
@@ -1101,17 +1092,17 @@
         <v>46280</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="47"/>
+      <c r="A12" s="49"/>
       <c r="B12" s="21">
         <f>B11+1</f>
         <v>8</v>
@@ -1124,16 +1115,16 @@
         <v>46282</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
+        <v>26</v>
+      </c>
+      <c r="F12" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="47"/>
+      <c r="H12" s="47"/>
     </row>
     <row r="13" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="48"/>
+      <c r="A13" s="50"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="11"/>
@@ -1143,7 +1134,7 @@
       <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="53">
+      <c r="A14" s="48">
         <v>5</v>
       </c>
       <c r="B14" s="15">
@@ -1158,18 +1149,18 @@
         <v>46287</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H14" s="19"/>
     </row>
     <row r="15" spans="1:8" ht="48" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
+      <c r="A15" s="49"/>
       <c r="B15" s="4">
         <f>B14+1</f>
         <v>10</v>
@@ -1182,18 +1173,18 @@
         <v>46289</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="H15" s="24"/>
     </row>
     <row r="16" spans="1:8" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="48"/>
+      <c r="A16" s="50"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
@@ -1201,11 +1192,11 @@
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="53">
+      <c r="A17" s="48">
         <v>6</v>
       </c>
       <c r="B17" s="15">
@@ -1220,17 +1211,17 @@
         <v>46294</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="32" x14ac:dyDescent="0.2">
-      <c r="A18" s="47"/>
+      <c r="A18" s="49"/>
       <c r="B18" s="4">
         <f>B17+1</f>
         <v>12</v>
@@ -1243,17 +1234,17 @@
         <v>46296</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="19" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="48"/>
+      <c r="A19" s="50"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="11"/>
@@ -1262,7 +1253,7 @@
       <c r="H19" s="25"/>
     </row>
     <row r="20" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="53">
+      <c r="A20" s="48">
         <v>7</v>
       </c>
       <c r="B20" s="15">
@@ -1277,18 +1268,18 @@
         <v>46301</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H20" s="18"/>
     </row>
     <row r="21" spans="1:9" ht="48" x14ac:dyDescent="0.2">
-      <c r="A21" s="47"/>
+      <c r="A21" s="49"/>
       <c r="B21" s="4">
         <f>B20+1</f>
         <v>14</v>
@@ -1301,28 +1292,28 @@
         <v>46303</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="22" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="48"/>
+      <c r="A22" s="50"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
-      <c r="F22" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="G22" s="54"/>
-      <c r="H22" s="54"/>
+      <c r="F22" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" s="51"/>
+      <c r="H22" s="51"/>
     </row>
     <row r="23" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="53">
+      <c r="A23" s="48">
         <v>8</v>
       </c>
       <c r="B23" s="15">
@@ -1337,7 +1328,7 @@
         <v>46308</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F23" s="18"/>
       <c r="G23" s="18"/>
@@ -1345,7 +1336,7 @@
       <c r="I23" s="8"/>
     </row>
     <row r="24" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="47"/>
+      <c r="A24" s="49"/>
       <c r="B24" s="4">
         <f>B23+1</f>
         <v>16</v>
@@ -1358,23 +1349,23 @@
         <v>46310</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H24" s="26"/>
     </row>
     <row r="25" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="48"/>
+      <c r="A25" s="50"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="11"/>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="14" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="53">
+      <c r="A26" s="48">
         <v>9</v>
       </c>
       <c r="B26" s="27">
@@ -1389,14 +1380,14 @@
         <v>46315</v>
       </c>
       <c r="E26" s="29" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F26" s="30"/>
       <c r="G26" s="30"/>
       <c r="H26" s="30"/>
     </row>
     <row r="27" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
+      <c r="A27" s="49"/>
       <c r="B27" s="4">
         <f>B26+1</f>
         <v>18</v>
@@ -1409,15 +1400,15 @@
         <v>46317</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H27" s="31"/>
     </row>
     <row r="28" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="48"/>
+      <c r="A28" s="50"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="11"/>
@@ -1427,7 +1418,7 @@
       <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="47">
+      <c r="A29" s="49">
         <v>10</v>
       </c>
       <c r="B29" s="15">
@@ -1442,12 +1433,12 @@
         <v>46322</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H29" s="9"/>
     </row>
     <row r="30" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="47"/>
+      <c r="A30" s="49"/>
       <c r="B30" s="4">
         <f>B29+1</f>
         <v>20</v>
@@ -1460,23 +1451,21 @@
         <v>46324</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="48"/>
+      <c r="A31" s="50"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
       <c r="D31" s="11"/>
       <c r="E31" s="32"/>
       <c r="F31" s="33"/>
       <c r="G31" s="33"/>
-      <c r="H31" s="56" t="s">
-        <v>67</v>
-      </c>
+      <c r="H31" s="34"/>
     </row>
     <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="47">
+      <c r="A32" s="49">
         <v>11</v>
       </c>
       <c r="B32" s="15">
@@ -1491,17 +1480,14 @@
         <v>46329</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="47"/>
+      <c r="A33" s="49"/>
       <c r="B33" s="4">
         <f>B32+1</f>
         <v>22</v>
@@ -1514,21 +1500,21 @@
         <v>46331</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="48"/>
+      <c r="A34" s="50"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="11"/>
       <c r="E34" s="32"/>
       <c r="F34" s="33"/>
       <c r="G34" s="33"/>
-      <c r="H34" s="56"/>
+      <c r="H34" s="34"/>
     </row>
     <row r="35" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="47">
+      <c r="A35" s="49">
         <v>12</v>
       </c>
       <c r="B35" s="15">
@@ -1543,12 +1529,12 @@
         <v>46336</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H35" s="9"/>
     </row>
     <row r="36" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="47"/>
+      <c r="A36" s="49"/>
       <c r="B36" s="4">
         <f>B35+1</f>
         <v>24</v>
@@ -1561,11 +1547,11 @@
         <v>46338</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="48"/>
+      <c r="A37" s="50"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
       <c r="D37" s="11"/>
@@ -1575,7 +1561,7 @@
       <c r="H37" s="34"/>
     </row>
     <row r="38" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="47">
+      <c r="A38" s="49">
         <v>13</v>
       </c>
       <c r="B38" s="15">
@@ -1590,12 +1576,12 @@
         <v>46343</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H38" s="9"/>
     </row>
     <row r="39" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" s="47"/>
+      <c r="A39" s="49"/>
       <c r="B39" s="4">
         <f>B38+1</f>
         <v>26</v>
@@ -1608,11 +1594,11 @@
         <v>46345</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" s="48"/>
+      <c r="A40" s="50"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
       <c r="D40" s="11"/>
@@ -1620,11 +1606,11 @@
       <c r="F40" s="33"/>
       <c r="G40" s="33"/>
       <c r="H40" s="25" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" s="51"/>
+      <c r="A41" s="54"/>
       <c r="B41" s="36"/>
       <c r="C41" s="35" t="s">
         <v>7</v>
@@ -1639,7 +1625,7 @@
       <c r="H41" s="39"/>
     </row>
     <row r="42" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="51"/>
+      <c r="A42" s="54"/>
       <c r="B42" s="35"/>
       <c r="C42" s="35" t="s">
         <v>11</v>
@@ -1649,14 +1635,14 @@
         <v>46352</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F42" s="39"/>
       <c r="G42" s="39"/>
       <c r="H42" s="41"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="52"/>
+      <c r="A43" s="55"/>
       <c r="B43" s="42"/>
       <c r="C43" s="42"/>
       <c r="D43" s="43"/>
@@ -1666,7 +1652,7 @@
       <c r="H43" s="46"/>
     </row>
     <row r="44" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="47">
+      <c r="A44" s="49">
         <v>14</v>
       </c>
       <c r="B44" s="15">
@@ -1681,12 +1667,12 @@
         <v>46357</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H44" s="9"/>
     </row>
     <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="47"/>
+      <c r="A45" s="49"/>
       <c r="B45" s="4">
         <f>B44+1</f>
         <v>28</v>
@@ -1699,11 +1685,11 @@
         <v>46359</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="48"/>
+      <c r="A46" s="50"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
       <c r="D46" s="11">
@@ -1716,7 +1702,7 @@
       <c r="H46" s="34"/>
     </row>
     <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" s="47">
+      <c r="A47" s="49">
         <v>15</v>
       </c>
       <c r="B47" s="15">
@@ -1731,14 +1717,14 @@
         <v>46364</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" s="47"/>
+      <c r="A48" s="49"/>
       <c r="B48" s="4">
         <f>B47+1</f>
         <v>30</v>
@@ -1751,14 +1737,14 @@
         <v>46366</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" s="48"/>
+      <c r="A49" s="50"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
       <c r="D49" s="11">
@@ -1771,7 +1757,7 @@
       <c r="H49" s="34"/>
     </row>
     <row r="50" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="47"/>
+      <c r="A50" s="49"/>
       <c r="B50" s="15"/>
       <c r="C50" s="4" t="s">
         <v>7</v>
@@ -1781,14 +1767,14 @@
         <v>46371</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H50" s="49" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="H50" s="52" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="47"/>
+      <c r="A51" s="49"/>
       <c r="C51" s="4" t="s">
         <v>11</v>
       </c>
@@ -1797,17 +1783,17 @@
         <v>46373</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="H51" s="50"/>
+        <v>61</v>
+      </c>
+      <c r="H51" s="53"/>
     </row>
     <row r="52" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="48"/>
+      <c r="A52" s="50"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F52" s="33"/>
       <c r="G52" s="33"/>
@@ -1815,18 +1801,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="F12:H12"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="A26:A28"/>
     <mergeCell ref="A50:A52"/>
     <mergeCell ref="H50:H51"/>
     <mergeCell ref="A32:A34"/>
@@ -1835,6 +1809,18 @@
     <mergeCell ref="A41:A43"/>
     <mergeCell ref="A44:A46"/>
     <mergeCell ref="A47:A49"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="A14:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>